<commit_message>
Re ultra mega final pa enviar
</commit_message>
<xml_diff>
--- a/datos_graficos.xlsx
+++ b/datos_graficos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USUARIO\Documents\WTF IS PROGRAMMING 2.0\UR CLASES\7_SEMESTRE\ICE\Proyecciones\ICE_Proyecciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC71D29B-77CB-4148-92A8-9E8940E3D8D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8646E398-0994-46D3-8247-146BEAF484CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{56B5A1B1-55DC-4A5A-A4D7-41B90A51D3EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{56B5A1B1-55DC-4A5A-A4D7-41B90A51D3EC}"/>
   </bookViews>
   <sheets>
     <sheet name="PIB" sheetId="1" r:id="rId1"/>
@@ -53,18 +53,6 @@
     <t>gasto 2</t>
   </si>
   <si>
-    <t>minero</t>
-  </si>
-  <si>
-    <t>minero 2</t>
-  </si>
-  <si>
-    <t>exportaciones</t>
-  </si>
-  <si>
-    <t>exportaciones 2</t>
-  </si>
-  <si>
     <t>año</t>
   </si>
   <si>
@@ -79,6 +67,18 @@
   <si>
     <t>Diferencia</t>
   </si>
+  <si>
+    <t>Sector Minero</t>
+  </si>
+  <si>
+    <t>Sector Minero  - Escenario Hipotético</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exportaciones </t>
+  </si>
+  <si>
+    <t>Exportaciones - Escenario Hipotético</t>
+  </si>
 </sst>
 </file>
 
@@ -87,7 +87,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000%"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,6 +96,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -124,9 +132,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -230,7 +239,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>minero</c:v>
+                  <c:v>Sector Minero</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -366,7 +375,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>minero 2</c:v>
+                  <c:v>Sector Minero  - Escenario Hipotético</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -502,7 +511,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>exportaciones</c:v>
+                  <c:v>Exportaciones </c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -638,7 +647,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>exportaciones 2</c:v>
+                  <c:v>Exportaciones - Escenario Hipotético</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1855,7 +1864,7 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B1">
         <v>2005</v>
@@ -2275,15 +2284,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7A9F8C1-8CA4-4141-BEB7-7F1CE9191F42}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="34.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B1">
         <v>2026</v>
@@ -2303,7 +2312,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1">
         <v>-4.7997234327583516E-2</v>
@@ -2323,7 +2332,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1">
         <v>0.12</v>
@@ -2343,7 +2352,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1">
         <v>1.116866779052017E-2</v>
@@ -2363,7 +2372,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1">
         <v>0.05</v>
@@ -2380,6 +2389,9 @@
       <c r="F5" s="1">
         <v>4.0135750351773081E-2</v>
       </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2394,7 +2406,7 @@
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B1">
         <v>2005</v>
@@ -2477,7 +2489,7 @@
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B2">
         <v>2185</v>
@@ -2560,7 +2572,7 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B3">
         <v>2185</v>

</xml_diff>